<commit_message>
Finalized core documentation and dated test execution results
</commit_message>
<xml_diff>
--- a/BookShelf-App/Docs/BookShelf_Test_Plan_And_Results.xlsx
+++ b/BookShelf-App/Docs/BookShelf_Test_Plan_And_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\BookShelf-App\BookShelf-App\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EFA4BD9-1A10-47B4-8407-69A79029CA37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28F605A-998C-4875-ACD9-2128B6685E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8160" yWindow="468" windowWidth="14892" windowHeight="11592" xr2:uid="{6F9BA980-EC11-4EDD-8B86-94156A86210F}"/>
   </bookViews>
@@ -38,12 +38,109 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+  <si>
+    <t>Test Case:</t>
+  </si>
+  <si>
+    <t>Description:</t>
+  </si>
+  <si>
+    <t>Date Executed:</t>
+  </si>
+  <si>
+    <t>RESULT:</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>TC-01</t>
+  </si>
+  <si>
+    <t>TC-02</t>
+  </si>
+  <si>
+    <t>TC-03</t>
+  </si>
+  <si>
+    <t>TC-04</t>
+  </si>
+  <si>
+    <t>TC-05</t>
+  </si>
+  <si>
+    <t>TC-06</t>
+  </si>
+  <si>
+    <t>TC-07</t>
+  </si>
+  <si>
+    <t>TC-08</t>
+  </si>
+  <si>
+    <t>TC-09</t>
+  </si>
+  <si>
+    <t>TC-10</t>
+  </si>
+  <si>
+    <t>Open Library API Remote Search</t>
+  </si>
+  <si>
+    <t>Fallback Cover Image Handling</t>
+  </si>
+  <si>
+    <t>Local SQLite CRUD Operations</t>
+  </si>
+  <si>
+    <t>Reading Status Persistence</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Validated live payload parsing.</t>
+  </si>
+  <si>
+    <t>Confirmed placeholder displays when cover_i is null.</t>
+  </si>
+  <si>
+    <t>Resolved index attribute issue; books save/delete cleanly.</t>
+  </si>
+  <si>
+    <t>Status picker updates SavedBooks table properly.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -57,7 +154,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,17 +162,75 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -86,6 +241,20 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C9164DCA-A4AC-49BB-B18F-7F14B46C98AA}" name="Table1" displayName="Table1" ref="B6:F23" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="B6:F23" xr:uid="{C9164DCA-A4AC-49BB-B18F-7F14B46C98AA}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{D15501BF-C621-4B86-82FA-53610D6B30A5}" name="Test Case:" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{46C21601-CF87-4B42-962F-3CE93A3C0A34}" name="Description:" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{44494DBF-0A21-40C9-B170-20656C11BD9C}" name="Date Executed:" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{FCFC73FD-F051-417E-A30C-2AF9968FD150}" name="RESULT:" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{B475B3F9-BEFF-4148-B74C-0C65F27CA0AF}" name="Notes:" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -405,9 +574,139 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{763BCA6D-F5EB-402F-AE4F-6747A12BB8EB}">
-  <dimension ref="A1"/>
+  <dimension ref="B5:F16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="14.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:6" s="2" customFormat="1" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="4">
+        <v>46261</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="4">
+        <v>46261</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="4">
+        <v>46261</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46261</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>